<commit_message>
SPM-84: re-read the Active events filters when the address changes
- Clicking a coordinator's name on the Coordinators tab now opens Active
  events filtered to them without a reload; the Active events tab clears
  the filters
- Add two page tests for both cases
- Add SPM-84-TC10 to the test case workbook and JSON
- Update the changelog and the traceability matrix
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-84_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-84_Test_Cases.xlsx
@@ -16,6 +16,7 @@
     <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -149,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,6 +178,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -886,6 +888,45 @@
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
     </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TC10</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>SPM-84-TC10</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Clicking a coordinator's name on the Coordinators tab opens the Active events list filtered to that coordinator, and the Active events tab clears the filter</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>AC4, AC7</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+    </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
@@ -983,7 +1024,8 @@
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>SPM-84-TC02</t>
+          <t>SPM-84-TC02
+SPM-84-TC10</t>
         </is>
       </c>
       <c r="F19" s="9" t="n"/>
@@ -1047,7 +1089,8 @@
       <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SPM-84-TC03
-SPM-84-TC04</t>
+SPM-84-TC04
+SPM-84-TC10</t>
         </is>
       </c>
       <c r="F22" s="9" t="n"/>
@@ -1368,6 +1411,213 @@
           <t>Actual Result</t>
         </is>
       </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: A dialog 'Reassign this event?' appears, saying Aisha Karim will no longer be able to manage it and that both coordinators are notified.
+Step 6: The message '"SPM84 Harbour Gala" has been reassigned from Aisha Karim to Benjamin Lau.' appears, and 'SPM84 Harbour Gala' leaves the list filtered to Aisha Karim.
+Step 7: Aisha Karim's 'Active events' count is now 2 and Benjamin Lau's is 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-84-TC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Clicking a coordinator's name on the Coordinators tab opens the Active events list filtered to that coordinator, and the Active events tab clears the filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>npm run fixtures:spm84 has been run (after SPM-84-TC09, run it again so SPM84 Harbour Gala is back with Aisha Karim). Aisha Karim holds three active events: SPM84 Harbour Gala (Planning), SPM84 Orchard Forum (Under review) and SPM84 Postponed Retreat (Postponed).
+Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Assignments' in the sidebar
+2. Click the 'Coordinators' tab
+3. Click 'Aisha Karim' in the Coordinator column
+4. Click the 'Active events' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Coordinator: Aisha Karim (3 active events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
+Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
       <c r="B12" s="3" t="n"/>
     </row>
     <row r="13">
@@ -1551,7 +1801,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
+Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
+Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1559,7 +1815,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1567,7 +1827,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1575,7 +1839,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1583,7 +1851,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1591,7 +1861,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1734,7 +2008,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1742,7 +2020,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1750,7 +2032,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1758,7 +2044,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1766,7 +2056,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1774,7 +2066,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1917,7 +2213,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1925,7 +2227,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1933,7 +2239,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1941,7 +2251,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1949,7 +2263,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1957,7 +2273,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2108,7 +2428,16 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The list offers 'Any status', then Submitted, Under review, Approved, Planning, Safety review, Safety approved, Confirmed and Postponed - no Draft, Rejected, Withdrawn, Cancelled or Completed.
+Step 5: Only 'SPM84 Harbour Gala' (Planning, Aisha Karim) is listed.
+Step 6: The page reopens on the 'Active events' tab with 'Aisha Karim' and 'Planning' still chosen, and still only 'SPM84 Harbour Gala' listed.
+Step 7: No rows are shown; the message 'No active events match these filters' appears with 'Try another coordinator or status.'
+Step 8: 'SPM84 Riverside Launch' (Confirmed, Benjamin Lau) is listed.
+Step 9: 'SPM84 Unassigned Request' is listed with Status 'Submitted' and Coordinator 'Not yet assigned', and an 'Assign to' control instead of 'Reassign to'.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2116,7 +2445,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2124,7 +2457,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2132,7 +2469,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2140,7 +2481,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2148,7 +2491,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2291,7 +2638,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: There is no 'Review request' button. Only the 'Change coordinator' card offers an action.
+Step 2: There is no 'Submit for safety check', 'Confirm event' or 'Edit event information' button, and no Venue, Equipment or Readiness tab.
+Step 4: The page shows 'Not authorised' and 'You don't have access to this event.'; no equipment can be added or changed.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2299,7 +2652,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2307,7 +2664,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2315,7 +2676,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2323,7 +2688,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2331,7 +2698,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2473,7 +2844,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: The top bar shows 'Clara Tay' and the role 'Event Coordinator'. The sidebar has no 'Assignments' link.
+Step 2: The Review Queue is empty and says 'Requests appear here once the Event Coordinator Lead assigns them to you.'
+Step 3: The 'Assignments' page shows 'You do not have access to this' and 'Assigning coordinators is the Event Coordinator Lead's role.' No coordinators or events are listed.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2481,7 +2858,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2489,7 +2870,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2497,7 +2882,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2505,7 +2894,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2513,7 +2904,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2664,7 +3059,15 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: 'You do not have access to this' and 'Assigning coordinators is the Event Coordinator Lead's role.' are shown; no events are listed.
+Step 4: The same refusal is shown for Technical Support; no events are listed.
+Step 6: The same refusal is shown for the Safety Officer; no events are listed.
+Step 8: The same refusal is shown for the Event Organiser; no coordinators are listed.
+Step 10: The same refusal is shown for the Attendee; no coordinators are listed.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2672,7 +3075,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2680,7 +3087,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2688,7 +3099,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2696,7 +3111,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2704,7 +3121,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2850,7 +3271,14 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: The 'Awaiting assignment' tab lists 'SPM84 Unassigned Request' with Client 'Meridian Financial Group'.
+Step 3: The message 'Clara Tay is now the coordinator for "SPM84 Unassigned Request". It has moved to Under review.' appears and the row leaves the Awaiting assignment list.
+Step 5: 'SPM84 Unassigned Request' is listed with Status 'Under review' and Coordinator 'Clara Tay'.
+Step 6: Clara Tay's 'Active events' count is now 1.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2858,7 +3286,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2866,7 +3298,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2874,7 +3310,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2882,7 +3322,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2890,7 +3332,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-84: record test case run
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-84_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-84_Test_Cases.xlsx
@@ -25,8 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1602,7 +1603,6 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1618,7 +1618,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
+Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1626,7 +1631,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1634,7 +1643,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1642,7 +1655,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1650,7 +1667,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1658,7 +1677,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>d66de75</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2083,7 +2106,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2276,6 +2299,86 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>d66de75</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2393,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2494,6 +2597,89 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The list offers 'Any status', then Submitted, Under review, Approved, Planning, Safety review, Safety approved, Confirmed and Postponed - no Draft, Rejected, Withdrawn, Cancelled or Completed.
+Step 5: Only 'SPM84 Harbour Gala' (Planning, Aisha Karim) is listed.
+Step 6: The page reopens on the 'Active events' tab with 'Aisha Karim' and 'Planning' still chosen, and still only 'SPM84 Harbour Gala' listed.
+Step 7: No rows are shown; the message 'No active events match these filters' appears with 'Try another coordinator or status.'
+Step 8: 'SPM84 Riverside Launch' (Confirmed, Benjamin Lau) is listed.
+Step 9: 'SPM84 Unassigned Request' is listed with Status 'Submitted' and Coordinator 'Not yet assigned', and an 'Assign to' control instead of 'Reassign to'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>d66de75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-84: Sammi's test run
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-84_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-84_Test_Cases.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TC01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TC02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TC03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TC04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TC05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TC06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -25,9 +25,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1279,7 +1278,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1397,6 +1396,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1477,6 +1477,83 @@
           <t>09f1efb</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: A dialog 'Reassign this event?' appears, saying Aisha Karim will no longer be able to manage it and that both coordinators are notified.
+Step 6: The message '"SPM84 Harbour Gala" has been reassigned from Aisha Karim to Benjamin Lau.' appears, and 'SPM84 Harbour Gala' leaves the list filtered to Aisha Karim.
+Step 7: Aisha Karim's 'Active events' count is now 2 and Benjamin Lau's is 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1484,623 +1561,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-84-TC10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Clicking a coordinator's name on the Coordinators tab opens the Active events list filtered to that coordinator, and the Active events tab clears the filter</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>npm run fixtures:spm84 has been run (after SPM-84-TC09, run it again so SPM84 Harbour Gala is back with Aisha Karim). Aisha Karim holds three active events: SPM84 Harbour Gala (Planning), SPM84 Orchard Forum (Under review) and SPM84 Postponed Retreat (Postponed).
-Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1. Click 'Assignments' in the sidebar
-2. Click the 'Coordinators' tab
-3. Click 'Aisha Karim' in the Coordinator column
-4. Click the 'Active events' tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Coordinator: Aisha Karim (3 active events)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="85" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
-Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
-Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Commit</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>d66de75</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-84-TC01</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>The Event Operations Manager is shown as the Event Coordinator Lead, with the same account, sidebar and Assignments screen as before</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>npm run fixtures:spm84 has been run.
-Grace Lim's account (grace.lim@connectsphere.com) is the role previously called Event Operations Manager.
-Logged out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1. Log in as grace.lim@connectsphere.com / password123
-2. Click 'Assignments' in the sidebar
-3. Click 'All Events' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Account: grace.lim@connectsphere.com / password123 (unchanged)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="125.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
-Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
-Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
-Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
-Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Commit</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>09f1efb</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-84-TC02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>The Coordinators tab lists every Event Coordinator with their number of active events, including one with none and a deactivated one who still holds an event</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>npm run fixtures:spm84 has been run. It creates four coordinator accounts of SPM-84's own:
-- Aisha Karim: SPM84 Harbour Gala (Planning), SPM84 Orchard Forum (Under review), SPM84 Postponed Retreat (Postponed) - active; SPM84 Closed Showcase (Completed), SPM84 Called Off Expo (Cancelled), SPM84 Rejected Request (Rejected), SPM84 Withdrawn Request (Withdrawn) - not active
-- Benjamin Lau: SPM84 Riverside Launch (Confirmed)
-- Clara Tay: SPM84 Past Seminar (Completed) only
-- Dennis Ho: account deactivated, still assigned SPM84 Inherited Workshop (Planning)
-Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1. Click 'Assignments' in the sidebar
-2. Click the 'Coordinators' tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Coordinators: Aisha Karim (3 active), Benjamin Lau (1), Clara Tay (0), Dennis Ho (1, account inactive)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="85" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Commit</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>09f1efb</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2129,7 +1589,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-84-TC03</t>
+          <t>SPM-84-TC10</t>
         </is>
       </c>
     </row>
@@ -2141,11 +1601,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The Active events tab, filtered to one coordinator, shows only their active events with coordinator, status, client and date, and each opens its event</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+          <t>Clicking a coordinator's name on the Coordinators tab opens the Active events list filtered to that coordinator, and the Active events tab clears the filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2153,12 +1613,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>npm run fixtures:spm84 has been run (Aisha Karim has three active and four inactive SPM84 events, all for the client Meridian Financial Group).
+          <t>npm run fixtures:spm84 has been run (after SPM-84-TC09, run it again so SPM84 Harbour Gala is back with Aisha Karim). Aisha Karim holds three active events: SPM84 Harbour Gala (Planning), SPM84 Orchard Forum (Under review) and SPM84 Postponed Retreat (Postponed).
 Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2167,13 +1627,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Assignments' in the sidebar
-2. Click the 'Active events' tab
-3. In 'Coordinator', choose 'Aisha Karim'
-4. Click 'SPM84 Harbour Gala'</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17.5" customHeight="1">
+2. Click the 'Coordinators' tab
+3. Click 'Aisha Karim' in the Coordinator column
+4. Click the 'Active events' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2181,11 +1641,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Coordinator filter: Aisha Karim</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="206.5" customHeight="1">
+          <t>Coordinator: Aisha Karim (3 active events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2193,9 +1653,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
-Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
-Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
+Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
         </is>
       </c>
     </row>
@@ -2221,6 +1680,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2238,9 +1698,8 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
-Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
-Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
+Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
         </is>
       </c>
     </row>
@@ -2298,7 +1757,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>09f1efb</t>
+          <t>d66de75</t>
         </is>
       </c>
     </row>
@@ -2309,6 +1768,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2318,9 +1778,8 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
-Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
-Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+          <t>Step 3: Without the page reloading, the 'Active events' tab is selected, 'Coordinator' shows 'Aisha Karim', 'Status' shows 'Any status', and only SPM84 Harbour Gala, SPM84 Orchard Forum and SPM84 Postponed Retreat are listed, each with Aisha Karim as the coordinator.
+Step 4: 'Coordinator' goes back to 'Any coordinator', and the list shows every active event again, including other coordinators' events (e.g. SPM84 Riverside Launch, Benjamin Lau).</t>
         </is>
       </c>
     </row>
@@ -2356,7 +1815,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Janelle</t>
+          <t>Sammi</t>
         </is>
       </c>
     </row>
@@ -2367,7 +1826,7 @@
         </is>
       </c>
       <c r="B24" s="15" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="25">
@@ -2376,18 +1835,14 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>d66de75</t>
-        </is>
-      </c>
+      <c r="B25" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2416,6 +1871,937 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
+          <t>SPM-84-TC01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The Event Operations Manager is shown as the Event Coordinator Lead, with the same account, sidebar and Assignments screen as before</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>npm run fixtures:spm84 has been run.
+Grace Lim's account (grace.lim@connectsphere.com) is the role previously called Event Operations Manager.
+Logged out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as grace.lim@connectsphere.com / password123
+2. Click 'Assignments' in the sidebar
+3. Click 'All Events' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Account: grace.lim@connectsphere.com / password123 (unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="125.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
+Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
+Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
+Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
+Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: Login succeeds with the existing password. The top bar shows 'Grace Lim' and the role 'Event Coordinator Lead' - not 'Operations Manager'. The sidebar shows Dashboard, Assignments, All Events, Venues and Notifications, as before.
+Step 2: The 'Assignments' page opens with three tabs: 'Awaiting assignment', 'Active events' and 'Coordinators'. 'Operations Manager' does not appear anywhere on the page.
+Step 3: The All Events list opens as before, with no 'Operations Manager' wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-84-TC02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The Coordinators tab lists every Event Coordinator with their number of active events, including one with none and a deactivated one who still holds an event</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>npm run fixtures:spm84 has been run. It creates four coordinator accounts of SPM-84's own:
+- Aisha Karim: SPM84 Harbour Gala (Planning), SPM84 Orchard Forum (Under review), SPM84 Postponed Retreat (Postponed) - active; SPM84 Closed Showcase (Completed), SPM84 Called Off Expo (Cancelled), SPM84 Rejected Request (Rejected), SPM84 Withdrawn Request (Withdrawn) - not active
+- Benjamin Lau: SPM84 Riverside Launch (Confirmed)
+- Clara Tay: SPM84 Past Seminar (Completed) only
+- Dennis Ho: account deactivated, still assigned SPM84 Inherited Workshop (Planning)
+Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Assignments' in the sidebar
+2. Click the 'Coordinators' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Coordinators: Aisha Karim (3 active), Benjamin Lau (1), Clara Tay (0), Dennis Ho (1, account inactive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table lists every Event Coordinator by name, A to Z, with an 'Active events' column. Aisha Karim shows 3 (her Completed, Cancelled, Rejected and Withdrawn events are not counted). Benjamin Lau shows 1. Clara Tay is listed with 0. Dennis Ho shows 1 and is labelled 'Account inactive'. The base coordinators (e.g. Daniel Tan, Priya Raj) are listed too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-84-TC03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The Active events tab, filtered to one coordinator, shows only their active events with coordinator, status, client and date, and each opens its event</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>npm run fixtures:spm84 has been run (Aisha Karim has three active and four inactive SPM84 events, all for the client Meridian Financial Group).
+Logged in as the Event Coordinator Lead, Grace Lim (grace.lim@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Assignments' in the sidebar
+2. Click the 'Active events' tab
+3. In 'Coordinator', choose 'Aisha Karim'
+4. Click 'SPM84 Harbour Gala'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Coordinator filter: Aisha Karim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="206.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>09f1efb</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>d66de75</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: A table of active events opens with the columns Event, Client, When, Status, Coordinator and 'Reassign to', and the filters 'Coordinator' (set to 'Any coordinator') and 'Status' (set to 'Any status').
+Step 3: Exactly three rows remain: 'SPM84 Harbour Gala' (Planning, 9 Nov 2027), 'SPM84 Orchard Forum' (Under review, 11 Nov 2027) and 'SPM84 Postponed Retreat' (Postponed, 16 Nov 2027), each with Client 'Meridian Financial Group' and Coordinator 'Aisha Karim'. SPM84 Closed Showcase, SPM84 Called Off Expo, SPM84 Rejected Request and SPM84 Withdrawn Request are not listed.
+Step 4: The event's Overview opens with the title 'SPM84 Harbour Gala', the status 'Planning', Coordinator 'Aisha Karim' and Company 'Meridian Financial Group', and a 'Change coordinator' card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
           <t>SPM-84-TC04</t>
         </is>
       </c>
@@ -2516,6 +2902,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2600,6 +2987,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -2682,6 +3070,85 @@
           <t>d66de75</t>
         </is>
       </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The list offers 'Any status', then Submitted, Under review, Approved, Planning, Safety review, Safety approved, Confirmed and Postponed - no Draft, Rejected, Withdrawn, Cancelled or Completed.
+Step 5: Only 'SPM84 Harbour Gala' (Planning, Aisha Karim) is listed.
+Step 6: The page reopens on the 'Active events' tab with 'Aisha Karim' and 'Planning' still chosen, and still only 'SPM84 Harbour Gala' listed.
+Step 7: No rows are shown; the message 'No active events match these filters' appears with 'Try another coordinator or status.'
+Step 8: 'SPM84 Riverside Launch' (Confirmed, Benjamin Lau) is listed.
+Step 9: 'SPM84 Unassigned Request' is listed with Status 'Submitted' and Coordinator 'Not yet assigned', and an 'Assign to' control instead of 'Reassign to'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2694,7 +3161,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2809,6 +3276,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2889,6 +3357,83 @@
           <t>09f1efb</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: There is no 'Review request' button. Only the 'Change coordinator' card offers an action.
+Step 2: There is no 'Submit for safety check', 'Confirm event' or 'Edit event information' button, and no Venue, Equipment or Readiness tab.
+Step 4: The page shows 'Not authorised' and 'You don't have access to this event.'; no equipment can be added or changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2901,7 +3446,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -3015,6 +3560,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3095,6 +3641,83 @@
           <t>09f1efb</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: The top bar shows 'Clara Tay' and the role 'Event Coordinator'. The sidebar has no 'Assignments' link.
+Step 2: The Review Queue is empty and says 'Requests appear here once the Event Coordinator Lead assigns them to you.'
+Step 3: The 'Assignments' page shows 'You do not have access to this' and 'Assigning coordinators is the Event Coordinator Lead's role.' No coordinators or events are listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3107,7 +3730,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -3230,6 +3853,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3312,6 +3936,85 @@
           <t>09f1efb</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: 'You do not have access to this' and 'Assigning coordinators is the Event Coordinator Lead's role.' are shown; no events are listed.
+Step 4: The same refusal is shown for Technical Support; no events are listed.
+Step 6: The same refusal is shown for the Safety Officer; no events are listed.
+Step 8: The same refusal is shown for the Event Organiser; no coordinators are listed.
+Step 10: The same refusal is shown for the Attendee; no coordinators are listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3324,7 +4027,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -3442,6 +4145,7 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3524,6 +4228,84 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: The 'Awaiting assignment' tab lists 'SPM84 Unassigned Request' with Client 'Meridian Financial Group'.
+Step 3: The message 'Clara Tay is now the coordinator for "SPM84 Unassigned Request". It has moved to Under review.' appears and the row leaves the Awaiting assignment list.
+Step 5: 'SPM84 Unassigned Request' is listed with Status 'Under review' and Coordinator 'Clara Tay'.
+Step 6: Clara Tay's 'Active events' count is now 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>